<commit_message>
format changes on prompt evaluation
</commit_message>
<xml_diff>
--- a/data/evaluation/Prompt Evaluation.xlsx
+++ b/data/evaluation/Prompt Evaluation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/data/evaluation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindpohl/Desktop/ReefGuide/rag_project_great_barrier_reef/data/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B94A200F-0A68-9840-B49F-0F774053E15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A6B9F2-2768-F54F-B0CA-77328D87FB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="520" yWindow="680" windowWidth="19280" windowHeight="16120" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
+    <workbookView xWindow="520" yWindow="740" windowWidth="28880" windowHeight="16120" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="71">
   <si>
     <t>Query</t>
   </si>
@@ -581,6 +581,9 @@
 vectors away from the equator and towards the poles.
 Specific to the GBRMP, increased frequency of mass coral bleaching events,
 threatening reef diversity, coral cover and ultimately reef eco-systems. (p. 57/58)</t>
+  </si>
+  <si>
+    <t>Average</t>
   </si>
 </sst>
 </file>
@@ -662,44 +665,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="12" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="12" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1069,66 +1072,66 @@
       <c r="C1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="O1" s="7" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="3">
         <v>5</v>
       </c>
       <c r="I2" s="8">
@@ -1137,46 +1140,46 @@
       <c r="J2" s="8">
         <v>2</v>
       </c>
-      <c r="K2" s="12">
+      <c r="K2" s="11">
         <f xml:space="preserve"> I2/H2</f>
         <v>0.4</v>
       </c>
-      <c r="L2" s="12">
+      <c r="L2" s="11">
         <f>IF(J2=0, "", I2/J2)</f>
         <v>1</v>
       </c>
       <c r="M2" s="8">
         <v>1</v>
       </c>
-      <c r="N2" s="14">
+      <c r="N2" s="12">
         <f>2*((K2*L2)/(K2+L2))</f>
         <v>0.57142857142857151</v>
       </c>
-      <c r="O2" s="1"/>
+      <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="3">
         <v>5</v>
       </c>
       <c r="I3" s="8">
@@ -1185,46 +1188,46 @@
       <c r="J3" s="8">
         <v>2</v>
       </c>
-      <c r="K3" s="12">
+      <c r="K3" s="11">
         <f t="shared" ref="K3:K13" si="0" xml:space="preserve"> I3/H3</f>
         <v>0.4</v>
       </c>
-      <c r="L3" s="12">
+      <c r="L3" s="11">
         <f t="shared" ref="L3:L16" si="1">IF(J3=0, "", I3/J3)</f>
         <v>1</v>
       </c>
       <c r="M3" s="8">
         <v>1</v>
       </c>
-      <c r="N3" s="14">
-        <f t="shared" ref="N3:N14" si="2">2*((K3*L3)/(K3+L3))</f>
+      <c r="N3" s="12">
+        <f t="shared" ref="N3:N13" si="2">2*((K3*L3)/(K3+L3))</f>
         <v>0.57142857142857151</v>
       </c>
-      <c r="O3" s="1"/>
+      <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="3">
         <v>5</v>
       </c>
       <c r="I4" s="8">
@@ -1233,46 +1236,46 @@
       <c r="J4" s="8">
         <v>2</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="11">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M4" s="8">
         <v>1</v>
       </c>
-      <c r="N4" s="14">
+      <c r="N4" s="12">
         <f t="shared" si="2"/>
         <v>0.57142857142857151</v>
       </c>
-      <c r="O4" s="1"/>
+      <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="10" t="s">
         <v>68</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="3">
         <v>5</v>
       </c>
       <c r="I5" s="8">
@@ -1281,46 +1284,46 @@
       <c r="J5" s="8">
         <v>2</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="11">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="L5" s="12">
+      <c r="L5" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M5" s="8">
         <v>1</v>
       </c>
-      <c r="N5" s="14">
+      <c r="N5" s="12">
         <f t="shared" si="2"/>
         <v>0.57142857142857151</v>
       </c>
-      <c r="O5" s="1"/>
+      <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="407" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="10" t="s">
         <v>31</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="3">
         <v>5</v>
       </c>
       <c r="I6" s="8">
@@ -1329,46 +1332,46 @@
       <c r="J6" s="8">
         <v>3</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="11">
         <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
-      <c r="L6" s="12">
+      <c r="L6" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M6" s="8">
         <v>1</v>
       </c>
-      <c r="N6" s="14">
+      <c r="N6" s="12">
         <f t="shared" si="2"/>
         <v>0.74999999999999989</v>
       </c>
-      <c r="O6" s="1"/>
+      <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" ht="119" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="3">
         <v>5</v>
       </c>
       <c r="I7" s="8">
@@ -1377,46 +1380,46 @@
       <c r="J7" s="8">
         <v>1</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="11">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M7" s="8">
         <v>1</v>
       </c>
-      <c r="N7" s="14">
+      <c r="N7" s="12">
         <f t="shared" si="2"/>
         <v>0.33333333333333337</v>
       </c>
-      <c r="O7" s="1"/>
+      <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="3">
         <v>5</v>
       </c>
       <c r="I8" s="8">
@@ -1425,46 +1428,46 @@
       <c r="J8" s="8">
         <v>1</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="11">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M8" s="8">
         <v>1</v>
       </c>
-      <c r="N8" s="14">
+      <c r="N8" s="12">
         <f t="shared" si="2"/>
         <v>0.33333333333333337</v>
       </c>
-      <c r="O8" s="1"/>
+      <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="3">
         <v>5</v>
       </c>
       <c r="I9" s="8">
@@ -1473,46 +1476,46 @@
       <c r="J9" s="8">
         <v>5</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="11">
         <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="11">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
       <c r="M9" s="8">
         <v>1</v>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="12">
         <f t="shared" si="2"/>
         <v>0.6</v>
       </c>
-      <c r="O9" s="1"/>
+      <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="85" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="10" t="s">
         <v>55</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="3">
         <v>5</v>
       </c>
       <c r="I10" s="8">
@@ -1521,43 +1524,43 @@
       <c r="J10" s="8">
         <v>1</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M10" s="8">
         <v>0</v>
       </c>
-      <c r="N10" s="15"/>
-      <c r="O10" s="1"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="2"/>
     </row>
     <row r="11" spans="1:15" ht="170" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="3">
         <v>5</v>
       </c>
       <c r="I11" s="8">
@@ -1566,46 +1569,46 @@
       <c r="J11" s="8">
         <v>1</v>
       </c>
-      <c r="K11" s="12">
+      <c r="K11" s="11">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M11" s="8">
         <v>1</v>
       </c>
-      <c r="N11" s="14">
+      <c r="N11" s="12">
         <f t="shared" si="2"/>
         <v>0.33333333333333337</v>
       </c>
-      <c r="O11" s="1"/>
+      <c r="O11" s="2"/>
     </row>
     <row r="12" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="3">
         <v>5</v>
       </c>
       <c r="I12" s="8">
@@ -1614,46 +1617,46 @@
       <c r="J12" s="8">
         <v>1</v>
       </c>
-      <c r="K12" s="12">
+      <c r="K12" s="11">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M12" s="8">
         <v>1</v>
       </c>
-      <c r="N12" s="14">
+      <c r="N12" s="12">
         <f t="shared" si="2"/>
         <v>0.33333333333333337</v>
       </c>
-      <c r="O12" s="1"/>
+      <c r="O12" s="2"/>
     </row>
     <row r="13" spans="1:15" ht="119" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="10" t="s">
         <v>54</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="3">
         <v>5</v>
       </c>
       <c r="I13" s="8">
@@ -1662,46 +1665,46 @@
       <c r="J13" s="8">
         <v>1</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="11">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="11">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M13" s="8">
         <v>1</v>
       </c>
-      <c r="N13" s="14">
+      <c r="N13" s="12">
         <f t="shared" si="2"/>
         <v>0.33333333333333337</v>
       </c>
-      <c r="O13" s="1"/>
+      <c r="O13" s="2"/>
     </row>
     <row r="14" spans="1:15" ht="85" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="3">
         <v>5</v>
       </c>
       <c r="I14" s="8">
@@ -1710,43 +1713,43 @@
       <c r="J14" s="8">
         <v>0</v>
       </c>
-      <c r="K14" s="12">
+      <c r="K14" s="11">
         <f xml:space="preserve"> I14/H14</f>
         <v>0</v>
       </c>
-      <c r="L14" s="13" t="str">
+      <c r="L14" s="15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="M14" s="8">
         <v>0</v>
       </c>
-      <c r="N14" s="15"/>
-      <c r="O14" s="1"/>
+      <c r="N14" s="14"/>
+      <c r="O14" s="2"/>
     </row>
     <row r="15" spans="1:15" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="3">
         <v>5</v>
       </c>
       <c r="I15" s="8">
@@ -1755,43 +1758,43 @@
       <c r="J15" s="8">
         <v>0</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="11">
         <f xml:space="preserve"> I15/H15</f>
         <v>0</v>
       </c>
-      <c r="L15" s="13" t="str">
+      <c r="L15" s="15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="M15" s="8">
         <v>0</v>
       </c>
-      <c r="N15" s="15"/>
-      <c r="O15" s="1"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="2"/>
     </row>
     <row r="16" spans="1:15" ht="102" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="10" t="s">
         <v>48</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="3">
         <v>5</v>
       </c>
       <c r="I16" s="8">
@@ -1800,69 +1803,73 @@
       <c r="J16" s="8">
         <v>0</v>
       </c>
-      <c r="K16" s="12">
+      <c r="K16" s="11">
         <f xml:space="preserve"> I16/H16</f>
         <v>0</v>
       </c>
-      <c r="L16" s="13" t="str">
+      <c r="L16" s="15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="M16" s="8">
         <v>0</v>
       </c>
-      <c r="N16" s="15"/>
-      <c r="O16" s="1"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="2"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="14">
+      <c r="A17" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="12">
         <f>AVERAGE(K2:K16)</f>
         <v>0.25333333333333341</v>
       </c>
-      <c r="L17" s="14">
+      <c r="L17" s="12">
         <f>AVERAGE(L2:L16)</f>
         <v>0.8833333333333333</v>
       </c>
-      <c r="M17" s="14">
+      <c r="M17" s="12">
         <f>AVERAGE(M2:M16)</f>
         <v>0.73333333333333328</v>
       </c>
-      <c r="N17" s="14">
+      <c r="N17" s="12">
         <f>AVERAGE(N2:N16)</f>
         <v>0.48203463203463204</v>
       </c>
-      <c r="O17" s="1"/>
+      <c r="O17" s="2"/>
       <c r="P17" s="1"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
       <c r="P18" s="1"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -1879,6 +1886,7 @@
       <c r="P19" s="2"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -1895,6 +1903,7 @@
       <c r="P20" s="2"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -1911,6 +1920,7 @@
       <c r="P21" s="2"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>

</xml_diff>